<commit_message>
Expand menu daily options to ten slots.
Save and load ten daily option recipes, include them in allergy exports, and commit the updated allergy form template with room for the extra rows.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/allergen-form-template.xlsx
+++ b/allergen-form-template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wesleynettleton/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wesleynettleton/Recipe Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B6E609D-8AB1-904C-A9D3-8C4809029BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41F0E4A-ED32-BB45-BDA7-5B422378C4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="20000" windowHeight="17500" activeTab="1" xr2:uid="{AEEE0734-66F7-2847-9B97-8BE0DB05D7DF}"/>
+    <workbookView xWindow="240" yWindow="600" windowWidth="20000" windowHeight="17400" activeTab="1" xr2:uid="{AEEE0734-66F7-2847-9B97-8BE0DB05D7DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Disclaimer" sheetId="2" r:id="rId1"/>
@@ -345,7 +345,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -371,15 +371,6 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
       <bottom style="thin">
         <color indexed="64"/>
@@ -390,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -405,7 +396,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -431,7 +421,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -468,9 +457,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1184,7 +1174,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="115.33203125" customWidth="1"/>
@@ -1192,65 +1182,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L1" s="28" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
+      <c r="L1" s="26" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="28"/>
-      <c r="M2" s="28"/>
-      <c r="N2" s="28"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
+      <c r="K2" s="25"/>
+      <c r="L2" s="26"/>
+      <c r="M2" s="26"/>
+      <c r="N2" s="26"/>
     </row>
     <row r="3" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
-      <c r="F3" s="27"/>
-      <c r="G3" s="27"/>
-      <c r="H3" s="27"/>
-      <c r="I3" s="27"/>
-      <c r="J3" s="27"/>
-      <c r="K3" s="27"/>
-      <c r="L3" s="28"/>
-      <c r="M3" s="28"/>
-      <c r="N3" s="28"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
     </row>
     <row r="4" spans="1:16" ht="8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="10"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="29"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="29"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="12"/>
+      <c r="L4" s="27"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="27"/>
     </row>
     <row r="5" spans="1:16" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2" t="e" vm="2">
@@ -1296,7 +1286,7 @@
       <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="25"/>
+      <c r="A6" s="23"/>
       <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
@@ -1338,356 +1328,356 @@
       </c>
     </row>
     <row r="7" spans="1:16" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
     </row>
     <row r="8" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="7"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="23"/>
-      <c r="N8" s="17"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="15"/>
     </row>
     <row r="9" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="7"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="P9" s="12"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="20"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="P9" s="11"/>
     </row>
     <row r="10" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A10" s="7"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
+      <c r="K10" s="15"/>
+      <c r="L10" s="15"/>
+      <c r="M10" s="15"/>
+      <c r="N10" s="15"/>
     </row>
     <row r="11" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="7"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="15"/>
+      <c r="M11" s="15"/>
+      <c r="N11" s="15"/>
     </row>
     <row r="12" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="7"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
     </row>
     <row r="13" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A13" s="7"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="22"/>
-      <c r="N13" s="17"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
+      <c r="K13" s="15"/>
+      <c r="L13" s="15"/>
+      <c r="M13" s="20"/>
+      <c r="N13" s="15"/>
     </row>
     <row r="14" spans="1:16" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="19"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+      <c r="M14" s="17"/>
+      <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A15" s="7"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="17"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+      <c r="L15" s="15"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="15"/>
     </row>
     <row r="16" spans="1:16" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A16" s="7"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="17"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="20"/>
+      <c r="K16" s="15"/>
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
     </row>
     <row r="17" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="7"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="20"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="15"/>
+      <c r="L17" s="15"/>
+      <c r="M17" s="15"/>
+      <c r="N17" s="15"/>
     </row>
     <row r="18" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A18" s="7"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
     </row>
     <row r="19" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="7"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
+      <c r="A19" s="6"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
+      <c r="K19" s="15"/>
+      <c r="L19" s="15"/>
+      <c r="M19" s="15"/>
+      <c r="N19" s="15"/>
     </row>
     <row r="20" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="7"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="20"/>
-      <c r="N20" s="17"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="18"/>
+      <c r="N20" s="15"/>
     </row>
     <row r="21" spans="1:14" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="19"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="17"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
+      <c r="M21" s="17"/>
+      <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A22" s="7"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="21"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="21"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="21"/>
+      <c r="A22" s="6"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="20"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="19"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="19"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="19"/>
     </row>
     <row r="23" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A23" s="7"/>
-      <c r="B23" s="21"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="21"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="21"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="21"/>
+      <c r="A23" s="6"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
     </row>
     <row r="24" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" s="7"/>
-      <c r="B24" s="21"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="21"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="21"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="21"/>
-      <c r="L24" s="21"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="22"/>
+      <c r="A24" s="6"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="20"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="19"/>
+      <c r="G24" s="19"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="19"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="20"/>
     </row>
     <row r="25" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="7"/>
-      <c r="B25" s="21"/>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
-      <c r="G25" s="21"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="21"/>
-      <c r="K25" s="21"/>
-      <c r="L25" s="21"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="21"/>
+      <c r="A25" s="6"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="19"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="19"/>
     </row>
     <row r="26" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26" s="7"/>
-      <c r="B26" s="21"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="21"/>
-      <c r="E26" s="21"/>
-      <c r="F26" s="21"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="21"/>
-      <c r="I26" s="21"/>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="22"/>
+      <c r="A26" s="6"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="20"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
+      <c r="G26" s="19"/>
+      <c r="H26" s="19"/>
+      <c r="I26" s="19"/>
+      <c r="J26" s="19"/>
+      <c r="K26" s="19"/>
+      <c r="L26" s="19"/>
+      <c r="M26" s="19"/>
+      <c r="N26" s="20"/>
     </row>
     <row r="27" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A27" s="7"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="21"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="21"/>
+      <c r="A27" s="6"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="20"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="20"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
+      <c r="L27" s="19"/>
+      <c r="M27" s="19"/>
+      <c r="N27" s="19"/>
     </row>
     <row r="28" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" s="14"/>
-      <c r="C28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="H28" s="15"/>
+      <c r="A28" s="13"/>
+      <c r="C28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="H28" s="14"/>
     </row>
     <row r="29" spans="1:14" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="24" t="s">
+      <c r="A29" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B29" s="2" t="e" vm="2">
@@ -1731,7 +1721,7 @@
       </c>
     </row>
     <row r="30" spans="1:14" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="25"/>
+      <c r="A30" s="23"/>
       <c r="B30" s="4" t="s">
         <v>1</v>
       </c>
@@ -1773,64 +1763,64 @@
       </c>
     </row>
     <row r="31" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="8" t="s">
+      <c r="A31" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="9"/>
-      <c r="C31" s="9"/>
-      <c r="D31" s="9"/>
-      <c r="E31" s="9"/>
-      <c r="F31" s="9"/>
-      <c r="G31" s="9"/>
-      <c r="H31" s="9"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
-      <c r="K31" s="9"/>
-      <c r="L31" s="9"/>
-      <c r="M31" s="9"/>
-      <c r="N31" s="9"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="8"/>
+      <c r="N31" s="8"/>
     </row>
     <row r="32" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="7"/>
+      <c r="A32" s="6"/>
       <c r="B32" s="3"/>
-      <c r="C32" s="22"/>
+      <c r="C32" s="20"/>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
-      <c r="F32" s="22"/>
+      <c r="F32" s="20"/>
       <c r="G32" s="3"/>
-      <c r="H32" s="22"/>
+      <c r="H32" s="20"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="22"/>
+      <c r="J32" s="20"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
-      <c r="N32" s="22"/>
+      <c r="N32" s="20"/>
     </row>
     <row r="33" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="7"/>
+      <c r="A33" s="6"/>
       <c r="B33" s="3"/>
-      <c r="C33" s="11"/>
+      <c r="C33" s="10"/>
       <c r="D33" s="3"/>
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
-      <c r="H33" s="22"/>
+      <c r="H33" s="20"/>
       <c r="I33" s="3"/>
       <c r="J33" s="3"/>
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
-      <c r="N33" s="22"/>
+      <c r="N33" s="20"/>
     </row>
     <row r="34" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="7"/>
+      <c r="A34" s="6"/>
       <c r="B34" s="3"/>
-      <c r="C34" s="22"/>
+      <c r="C34" s="20"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
-      <c r="H34" s="22"/>
+      <c r="H34" s="20"/>
       <c r="I34" s="3"/>
       <c r="J34" s="3"/>
       <c r="K34" s="3"/>
@@ -1839,7 +1829,7 @@
       <c r="N34" s="3"/>
     </row>
     <row r="35" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="7"/>
+      <c r="A35" s="6"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -1855,14 +1845,14 @@
       <c r="N35" s="3"/>
     </row>
     <row r="36" spans="1:14" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="7"/>
+      <c r="A36" s="6"/>
       <c r="B36" s="3"/>
-      <c r="C36" s="22"/>
+      <c r="C36" s="20"/>
       <c r="D36" s="3"/>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
-      <c r="H36" s="22"/>
+      <c r="H36" s="20"/>
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
       <c r="K36" s="3"/>
@@ -1871,14 +1861,14 @@
       <c r="N36" s="3"/>
     </row>
     <row r="37" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" s="7"/>
+      <c r="A37" s="6"/>
       <c r="B37" s="3"/>
-      <c r="C37" s="22"/>
+      <c r="C37" s="20"/>
       <c r="D37" s="3"/>
-      <c r="E37" s="22"/>
+      <c r="E37" s="20"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
-      <c r="H37" s="22"/>
+      <c r="H37" s="20"/>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
       <c r="K37" s="3"/>
@@ -1887,75 +1877,75 @@
       <c r="N37" s="3"/>
     </row>
     <row r="38" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-      <c r="I38" s="9"/>
-      <c r="J38" s="9"/>
-      <c r="K38" s="9"/>
-      <c r="L38" s="9"/>
-      <c r="M38" s="9"/>
-      <c r="N38" s="9"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
     </row>
     <row r="39" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" s="7"/>
+      <c r="A39" s="6"/>
       <c r="B39" s="3"/>
-      <c r="C39" s="22"/>
+      <c r="C39" s="20"/>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
-      <c r="F39" s="22"/>
+      <c r="F39" s="20"/>
       <c r="G39" s="3"/>
-      <c r="H39" s="22"/>
+      <c r="H39" s="20"/>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
-      <c r="M39" s="22"/>
-      <c r="N39" s="22"/>
+      <c r="M39" s="20"/>
+      <c r="N39" s="20"/>
     </row>
     <row r="40" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" s="7"/>
+      <c r="A40" s="6"/>
       <c r="B40" s="3"/>
-      <c r="C40" s="22"/>
+      <c r="C40" s="20"/>
       <c r="D40" s="3"/>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
-      <c r="H40" s="22"/>
+      <c r="H40" s="20"/>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
-      <c r="M40" s="11"/>
-      <c r="N40" s="11"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
     </row>
     <row r="41" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" s="7"/>
+      <c r="A41" s="6"/>
       <c r="B41" s="3"/>
-      <c r="C41" s="22"/>
+      <c r="C41" s="20"/>
       <c r="D41" s="3"/>
-      <c r="E41" s="22"/>
+      <c r="E41" s="20"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
-      <c r="H41" s="22"/>
+      <c r="H41" s="20"/>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
-      <c r="M41" s="22"/>
+      <c r="M41" s="20"/>
       <c r="N41" s="3"/>
     </row>
     <row r="42" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" s="7"/>
+      <c r="A42" s="6"/>
       <c r="B42" s="3"/>
-      <c r="C42" s="22"/>
+      <c r="C42" s="20"/>
       <c r="D42" s="3"/>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
@@ -1969,9 +1959,9 @@
       <c r="N42" s="3"/>
     </row>
     <row r="43" spans="1:14" ht="54" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" s="7"/>
+      <c r="A43" s="6"/>
       <c r="B43" s="3"/>
-      <c r="C43" s="22"/>
+      <c r="C43" s="20"/>
       <c r="D43" s="3"/>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -1982,17 +1972,17 @@
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
-      <c r="N43" s="22"/>
+      <c r="N43" s="20"/>
     </row>
     <row r="44" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" s="7"/>
+      <c r="A44" s="6"/>
       <c r="B44" s="3"/>
-      <c r="C44" s="22"/>
+      <c r="C44" s="20"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
-      <c r="H44" s="22"/>
+      <c r="H44" s="20"/>
       <c r="I44" s="3"/>
       <c r="J44" s="3"/>
       <c r="K44" s="3"/>
@@ -2001,41 +1991,41 @@
       <c r="N44" s="3"/>
     </row>
     <row r="45" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="8" t="s">
+      <c r="A45" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
-      <c r="G45" s="9"/>
-      <c r="H45" s="9"/>
-      <c r="I45" s="9"/>
-      <c r="J45" s="9"/>
-      <c r="K45" s="9"/>
-      <c r="L45" s="9"/>
-      <c r="M45" s="9"/>
-      <c r="N45" s="9"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8"/>
+      <c r="H45" s="8"/>
+      <c r="I45" s="8"/>
+      <c r="J45" s="8"/>
+      <c r="K45" s="8"/>
+      <c r="L45" s="8"/>
+      <c r="M45" s="8"/>
+      <c r="N45" s="8"/>
     </row>
     <row r="46" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="7"/>
+      <c r="A46" s="6"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="11"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
       <c r="G46" s="3"/>
-      <c r="H46" s="11"/>
+      <c r="H46" s="10"/>
       <c r="I46" s="3"/>
-      <c r="J46" s="11"/>
+      <c r="J46" s="10"/>
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
       <c r="N46" s="3"/>
     </row>
     <row r="47" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="7"/>
+      <c r="A47" s="6"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -2051,14 +2041,14 @@
       <c r="N47" s="3"/>
     </row>
     <row r="48" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="7"/>
+      <c r="A48" s="6"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
-      <c r="H48" s="11"/>
+      <c r="H48" s="10"/>
       <c r="I48" s="3"/>
       <c r="J48" s="3"/>
       <c r="K48" s="3"/>
@@ -2067,7 +2057,7 @@
       <c r="N48" s="3"/>
     </row>
     <row r="49" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="7"/>
+      <c r="A49" s="6"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -2082,15 +2072,101 @@
       <c r="M49" s="3"/>
       <c r="N49" s="3"/>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="K50" s="16"/>
-      <c r="L50" s="16"/>
-      <c r="M50" s="16"/>
-      <c r="N50" s="16"/>
-    </row>
-    <row r="52" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="6"/>
-      <c r="F52" s="6"/>
+    <row r="50" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+    </row>
+    <row r="51" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+    </row>
+    <row r="52" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="28"/>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+    </row>
+    <row r="53" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+      <c r="J53" s="3"/>
+      <c r="K53" s="3"/>
+      <c r="L53" s="3"/>
+      <c r="M53" s="3"/>
+      <c r="N53" s="3"/>
+    </row>
+    <row r="54" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="3"/>
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+      <c r="J54" s="3"/>
+      <c r="K54" s="3"/>
+      <c r="L54" s="3"/>
+      <c r="M54" s="3"/>
+      <c r="N54" s="3"/>
+    </row>
+    <row r="55" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="3"/>
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="3"/>
+      <c r="I55" s="3"/>
+      <c r="J55" s="3"/>
+      <c r="K55" s="3"/>
+      <c r="L55" s="3"/>
+      <c r="M55" s="3"/>
+      <c r="N55" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -2105,12 +2181,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="852e583b-9710-4529-bad4-560af3684856">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1eba3e3f-0465-4954-b816-13c76d16a087" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2343,20 +2421,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="852e583b-9710-4529-bad4-560af3684856">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1eba3e3f-0465-4954-b816-13c76d16a087" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF882E8C-234C-4AE9-BF8D-472CEC75E993}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="852e583b-9710-4529-bad4-560af3684856"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1eba3e3f-0465-4954-b816-13c76d16a087"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2381,18 +2466,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF882E8C-234C-4AE9-BF8D-472CEC75E993}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="852e583b-9710-4529-bad4-560af3684856"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1eba3e3f-0465-4954-b816-13c76d16a087"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update allergy export template formatting.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/allergen-form-template.xlsx
+++ b/allergen-form-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wesleynettleton/Recipe Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D41F0E4A-ED32-BB45-BDA7-5B422378C4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA738A83-B968-7842-BEF6-DBBE58CF3315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="600" windowWidth="20000" windowHeight="17400" activeTab="1" xr2:uid="{AEEE0734-66F7-2847-9B97-8BE0DB05D7DF}"/>
   </bookViews>
@@ -264,7 +264,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -330,6 +330,12 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="22"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -381,7 +387,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -442,6 +448,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -460,7 +467,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1182,46 +1191,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L1" s="26" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
+      <c r="L1" s="27" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
+      <c r="L2" s="27"/>
+      <c r="M2" s="27"/>
+      <c r="N2" s="27"/>
     </row>
     <row r="3" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="26"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
+      <c r="J3" s="26"/>
+      <c r="K3" s="26"/>
+      <c r="L3" s="27"/>
+      <c r="M3" s="27"/>
+      <c r="N3" s="27"/>
     </row>
     <row r="4" spans="1:16" ht="8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="9"/>
@@ -1235,12 +1244,12 @@
       <c r="I4" s="12"/>
       <c r="J4" s="12"/>
       <c r="K4" s="12"/>
-      <c r="L4" s="27"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="27"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="28"/>
+      <c r="N4" s="28"/>
     </row>
     <row r="5" spans="1:16" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2" t="e" vm="2">
@@ -1286,7 +1295,7 @@
       <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="23"/>
+      <c r="A6" s="24"/>
       <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
@@ -1677,7 +1686,7 @@
       <c r="H28" s="14"/>
     </row>
     <row r="29" spans="1:14" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="23" t="s">
         <v>0</v>
       </c>
       <c r="B29" s="2" t="e" vm="2">
@@ -1721,7 +1730,7 @@
       </c>
     </row>
     <row r="30" spans="1:14" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="23"/>
+      <c r="A30" s="24"/>
       <c r="B30" s="4" t="s">
         <v>1</v>
       </c>
@@ -2009,7 +2018,7 @@
       <c r="N45" s="8"/>
     </row>
     <row r="46" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="6"/>
+      <c r="A46" s="29"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
@@ -2025,7 +2034,7 @@
       <c r="N46" s="3"/>
     </row>
     <row r="47" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="6"/>
+      <c r="A47" s="29"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -2041,7 +2050,7 @@
       <c r="N47" s="3"/>
     </row>
     <row r="48" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="6"/>
+      <c r="A48" s="29"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
@@ -2057,7 +2066,7 @@
       <c r="N48" s="3"/>
     </row>
     <row r="49" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="6"/>
+      <c r="A49" s="29"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -2073,7 +2082,7 @@
       <c r="N49" s="3"/>
     </row>
     <row r="50" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="3"/>
+      <c r="A50" s="29"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
@@ -2089,7 +2098,7 @@
       <c r="N50" s="3"/>
     </row>
     <row r="51" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="3"/>
+      <c r="A51" s="29"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -2105,12 +2114,12 @@
       <c r="N51" s="3"/>
     </row>
     <row r="52" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="28"/>
+      <c r="A52" s="29"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
       <c r="E52" s="3"/>
-      <c r="F52" s="28"/>
+      <c r="F52" s="22"/>
       <c r="G52" s="3"/>
       <c r="H52" s="3"/>
       <c r="I52" s="3"/>
@@ -2121,7 +2130,7 @@
       <c r="N52" s="3"/>
     </row>
     <row r="53" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="3"/>
+      <c r="A53" s="29"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -2137,7 +2146,7 @@
       <c r="N53" s="3"/>
     </row>
     <row r="54" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="3"/>
+      <c r="A54" s="29"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
@@ -2153,7 +2162,7 @@
       <c r="N54" s="3"/>
     </row>
     <row r="55" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="3"/>
+      <c r="A55" s="29"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
@@ -2181,14 +2190,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="852e583b-9710-4529-bad4-560af3684856">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="1eba3e3f-0465-4954-b816-13c76d16a087" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2421,27 +2428,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="852e583b-9710-4529-bad4-560af3684856">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="1eba3e3f-0465-4954-b816-13c76d16a087" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF882E8C-234C-4AE9-BF8D-472CEC75E993}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="852e583b-9710-4529-bad4-560af3684856"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1eba3e3f-0465-4954-b816-13c76d16a087"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2466,9 +2466,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF882E8C-234C-4AE9-BF8D-472CEC75E993}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="852e583b-9710-4529-bad4-560af3684856"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1eba3e3f-0465-4954-b816-13c76d16a087"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update allergy export template for per-day Baguette slot.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/allergen-form-template.xlsx
+++ b/allergen-form-template.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wesleynettleton/Recipe Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA738A83-B968-7842-BEF6-DBBE58CF3315}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A088C3D-A0D1-A44F-984B-1473D0E1C18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="600" windowWidth="20000" windowHeight="17400" activeTab="1" xr2:uid="{AEEE0734-66F7-2847-9B97-8BE0DB05D7DF}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="1" xr2:uid="{AEEE0734-66F7-2847-9B97-8BE0DB05D7DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Disclaimer" sheetId="2" r:id="rId1"/>
     <sheet name="Allergens" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Allergens!$A$1:$N$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Allergens!$A$1:$N$55</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -449,6 +449,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -466,9 +469,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1191,46 +1191,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="L1" s="27" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
+      <c r="L1" s="28" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="27"/>
-      <c r="M2" s="27"/>
-      <c r="N2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+      <c r="L2" s="28"/>
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
     </row>
     <row r="3" spans="1:16" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="27"/>
-      <c r="N3" s="27"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27"/>
+      <c r="J3" s="27"/>
+      <c r="K3" s="27"/>
+      <c r="L3" s="28"/>
+      <c r="M3" s="28"/>
+      <c r="N3" s="28"/>
     </row>
     <row r="4" spans="1:16" ht="8" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="9"/>
@@ -1244,12 +1244,12 @@
       <c r="I4" s="12"/>
       <c r="J4" s="12"/>
       <c r="K4" s="12"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="28"/>
-      <c r="N4" s="28"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="29"/>
     </row>
     <row r="5" spans="1:16" ht="37" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="24" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="2" t="e" vm="2">
@@ -1295,7 +1295,7 @@
       <c r="P5" s="1"/>
     </row>
     <row r="6" spans="1:16" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
+      <c r="A6" s="25"/>
       <c r="B6" s="4" t="s">
         <v>1</v>
       </c>
@@ -1686,7 +1686,7 @@
       <c r="H28" s="14"/>
     </row>
     <row r="29" spans="1:14" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="23" t="s">
+      <c r="A29" s="24" t="s">
         <v>0</v>
       </c>
       <c r="B29" s="2" t="e" vm="2">
@@ -1730,7 +1730,7 @@
       </c>
     </row>
     <row r="30" spans="1:14" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="24"/>
+      <c r="A30" s="25"/>
       <c r="B30" s="4" t="s">
         <v>1</v>
       </c>
@@ -2018,7 +2018,7 @@
       <c r="N45" s="8"/>
     </row>
     <row r="46" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" s="29"/>
+      <c r="A46" s="23"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
@@ -2034,7 +2034,7 @@
       <c r="N46" s="3"/>
     </row>
     <row r="47" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="29"/>
+      <c r="A47" s="23"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
@@ -2050,7 +2050,7 @@
       <c r="N47" s="3"/>
     </row>
     <row r="48" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" s="29"/>
+      <c r="A48" s="23"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
       <c r="D48" s="3"/>
@@ -2066,7 +2066,7 @@
       <c r="N48" s="3"/>
     </row>
     <row r="49" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="29"/>
+      <c r="A49" s="23"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
       <c r="D49" s="3"/>
@@ -2082,7 +2082,7 @@
       <c r="N49" s="3"/>
     </row>
     <row r="50" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="29"/>
+      <c r="A50" s="23"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
       <c r="D50" s="3"/>
@@ -2098,7 +2098,7 @@
       <c r="N50" s="3"/>
     </row>
     <row r="51" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="29"/>
+      <c r="A51" s="23"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
       <c r="D51" s="3"/>
@@ -2114,7 +2114,7 @@
       <c r="N51" s="3"/>
     </row>
     <row r="52" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="29"/>
+      <c r="A52" s="23"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
       <c r="D52" s="3"/>
@@ -2130,7 +2130,7 @@
       <c r="N52" s="3"/>
     </row>
     <row r="53" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="29"/>
+      <c r="A53" s="23"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
       <c r="D53" s="3"/>
@@ -2146,7 +2146,7 @@
       <c r="N53" s="3"/>
     </row>
     <row r="54" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="29"/>
+      <c r="A54" s="23"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
       <c r="D54" s="3"/>
@@ -2162,7 +2162,7 @@
       <c r="N54" s="3"/>
     </row>
     <row r="55" spans="1:14" ht="55" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="29"/>
+      <c r="A55" s="23"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
       <c r="D55" s="3"/>
@@ -2185,20 +2185,11 @@
     <mergeCell ref="L1:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="42" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" scale="37" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CAD302C731784944A76C557646D1390A" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="606f697e215d3216815275764e1ab89e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="852e583b-9710-4529-bad4-560af3684856" xmlns:ns3="1eba3e3f-0465-4954-b816-13c76d16a087" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3cb8afb69c30e61a29255a33187e150a" ns2:_="" ns3:_="">
     <xsd:import namespace="852e583b-9710-4529-bad4-560af3684856"/>
@@ -2427,6 +2418,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2439,14 +2439,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C27DBB0D-4CD5-4B73-96D0-648DDE44DECB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2461,6 +2453,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Refine allergy export template formatting.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/allergen-form-template.xlsx
+++ b/allergen-form-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wesleynettleton/Recipe Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A088C3D-A0D1-A44F-984B-1473D0E1C18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C39CF3C3-F328-1D4A-A725-57713A15511B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="33600" windowHeight="21000" activeTab="1" xr2:uid="{AEEE0734-66F7-2847-9B97-8BE0DB05D7DF}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="20400" activeTab="1" xr2:uid="{AEEE0734-66F7-2847-9B97-8BE0DB05D7DF}"/>
   </bookViews>
   <sheets>
     <sheet name="Disclaimer" sheetId="2" r:id="rId1"/>
@@ -1180,9 +1180,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{494ACDF7-CD43-F44E-A7FF-E0FCB95B861B}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
   <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2185,7 +2182,10 @@
     <mergeCell ref="L1:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="37" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" scale="35" fitToHeight="2" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="28" max="13" man="1"/>
+  </rowBreaks>
 </worksheet>
 </file>
 
@@ -2419,15 +2419,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="852e583b-9710-4529-bad4-560af3684856">
@@ -2436,6 +2427,15 @@
     <TaxCatchAll xmlns="1eba3e3f-0465-4954-b816-13c76d16a087" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2458,14 +2458,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BF882E8C-234C-4AE9-BF8D-472CEC75E993}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
@@ -2480,4 +2472,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D164A66A-8184-4E5E-8C43-D54D8590D4C3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>